<commit_message>
Add new Excel reports for April 24, 2026
- Created Report_20260424_084324.xlsx with multiple worksheets and styles.
- Created Report_20260424_084532.xlsx with similar structure and content.
</commit_message>
<xml_diff>
--- a/data/output/westmarket.xlsx
+++ b/data/output/westmarket.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,45 @@
       </c>
       <c r="C2" t="n">
         <v>57.14285714285714</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update folder structure and remove obsolete data files
</commit_message>
<xml_diff>
--- a/data/output/westmarket.xlsx
+++ b/data/output/westmarket.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,45 +446,6 @@
         <v>57.14285714285714</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" t="n">
-        <v>60</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new Excel files for YTD data updates
- Created YTD_20260424_095639.xlsx with updated data.
- Created YTD_20260424_095750.xlsx with additional data.
</commit_message>
<xml_diff>
--- a/data/output/westmarket.xlsx
+++ b/data/output/westmarket.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="westmarket" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -444,6 +444,45 @@
       </c>
       <c r="C2" t="n">
         <v>57.14285714285714</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="n">
+        <v>57.14285714285714</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>57.14285714285714</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>85.71428571428571</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update README for clarity and enhance .gitignore; add new output Excel file
</commit_message>
<xml_diff>
--- a/data/output/westmarket.xlsx
+++ b/data/output/westmarket.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="westmarket" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,6 +511,19 @@
         <v>57.14285714285714</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>42.85714285714285</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>